<commit_message>
Deliverables: work in progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qy8CbYD8GTpf6MSCs4mucy
</commit_message>
<xml_diff>
--- a/deliverables/greek_banking_model.xlsx
+++ b/deliverables/greek_banking_model.xlsx
@@ -6116,14 +6116,14 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="39" t="inlineStr">
         <is>
-          <t>DTC = deferred tax credits: a tax claim on the Greek State that counts in CET1 capital. ECB funding is the amount due to the ECB and central banks at year end (data/manual/ecb_funding.csv, report and page in that file); all of the 2024 amount is Alpha's.</t>
+          <t>DTC = deferred tax credits: a tax claim on the Greek State that counts in CET1 capital. ECB funding is the amount due to the ECB and central banks at year end (02_Banking_Sector_Dashboard/data/manual/ecb_funding.csv, report and page in that file); all of the 2024 amount is Alpha's.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>2. NII RATE AND VOLUME WALK, 2022 TO 2023 (€m)</t>
+          <t>2A. NII RATE AND VOLUME WALK, 2022 TO 2023 (€m)</t>
         </is>
       </c>
     </row>
@@ -6252,7 +6252,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>2. NII RATE AND VOLUME WALK, 2023 TO 2024 (€m)</t>
+          <t>2B. NII RATE AND VOLUME WALK, 2023 TO 2024 (€m)</t>
         </is>
       </c>
     </row>
@@ -6691,7 +6691,7 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="39" t="inlineStr">
         <is>
-          <t>Three-year adverse scenario on the 31.12.2022 balance sheet, as reported by each bank (data/manual/eba_stress_test_2023.csv). Not comparable with the simplified one-year test above.</t>
+          <t>Three-year adverse scenario on the 31.12.2022 balance sheet, as reported by each bank (02_Banking_Sector_Dashboard/data/manual/eba_stress_test_2023.csv). Not comparable with the simplified one-year test above.</t>
         </is>
       </c>
     </row>
@@ -7052,6 +7052,10 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <rowBreaks count="2" manualBreakCount="2">
+    <brk id="28" min="0" max="16383" man="1"/>
+    <brk id="53" min="0" max="16383" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
 
@@ -7394,7 +7398,7 @@
       </c>
       <c r="D27" s="85" t="inlineStr">
         <is>
-          <t>Earning assets fall by the same amount</t>
+          <t>Loans fall by 15%. Average total assets fall by the same euro amount</t>
         </is>
       </c>
     </row>
@@ -7443,7 +7447,7 @@
         </is>
       </c>
       <c r="B30" s="86" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C30" s="86" t="inlineStr">
         <is>
@@ -7452,7 +7456,7 @@
       </c>
       <c r="D30" s="84" t="inlineStr">
         <is>
-          <t>On the change in profit</t>
+          <t>Applied to the change in profit before tax</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7798,7 @@
       <c r="C56" s="13" t="n"/>
       <c r="D56" s="14" t="n"/>
     </row>
-    <row r="57" ht="16" customHeight="1">
+    <row r="57" ht="17.5" customHeight="1">
       <c r="A57" s="28" t="inlineStr">
         <is>
           <t>CET1 ratios</t>
@@ -7802,7 +7806,7 @@
       </c>
       <c r="B57" s="85" t="inlineStr">
         <is>
-          <t>Banks treat dividend accruals differently</t>
+          <t>Include year-end profit net of the dividend accrual that each bank applies, so they are not perfectly comparable</t>
         </is>
       </c>
       <c r="C57" s="13" t="n"/>

</xml_diff>

<commit_message>
Deliverables rebuilt from the verified dataset; notebook builder in sync; CET1 dividend note per bank; CoE line 10%; plain separators in app titles
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qy8CbYD8GTpf6MSCs4mucy
</commit_message>
<xml_diff>
--- a/deliverables/greek_banking_model.xlsx
+++ b/deliverables/greek_banking_model.xlsx
@@ -2282,7 +2282,7 @@
       <c r="F25" s="23" t="n">
         <v>2600</v>
       </c>
-      <c r="G25" s="24" t="n">
+      <c r="G25" s="25" t="n">
         <v>2400</v>
       </c>
       <c r="H25" s="23" t="n">
@@ -2366,7 +2366,7 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="39" t="inlineStr">
         <is>
-          <t>Green = best of the four banks in 2024 (highest, or lowest for cost-to-income, cost of risk, NPE ratio, DTC and DTC share of CET1). Size items and the loan-to-deposit ratio are not ranked. Sector columns show the sum of the four banks for amounts only.</t>
+          <t>Green = best of the four banks in 2024 (highest, or lowest for cost-to-income, cost of risk, NPE ratio and DTC share of CET1). Amounts that depend on size (loans, deposits, total assets, equity, DTC) and the loan-to-deposit ratio are not ranked. Sector columns show the sum of the four banks for amounts only.</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6591,7 @@
     <row r="44" ht="43.5" customHeight="1">
       <c r="A44" s="39" t="inlineStr">
         <is>
-          <t>Shocks: +200bp cost of risk, −15% loans, −50bp NIM. Costs flat, 29% tax on the change in profit, no dividends, RWAs unchanged. CET1 at the end of the stress year = (reported CET1 ratio × RWAs + stressed net profit) / RWAs. A bank that stays profitable ends the year with more CET1 because no dividend is paid. Extra cost of risk before a pre-tax loss = FY2024 profit before tax / loans. Simplified, static, one year: directional only.</t>
+          <t>Shocks: cost of risk up 200bp, loans down 15%, NIM down 50bp. Costs flat, 29% tax on the change in profit, no dividends, RWAs unchanged. CET1 at the end of the stress year = (reported CET1 ratio × RWAs + stressed net profit) / RWAs. A bank that stays profitable ends the year with more CET1 because no dividend is paid. Extra cost of risk before a pre-tax loss = FY2024 profit before tax / loans. Simplified, static, one year: directional only.</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="39" t="inlineStr">
         <is>
-          <t>Justified P/TBV = (RoTE − g) / (CoE − g), with CoE 10% and g 2% as stated assumptions. No market prices are used. A bank that earns exactly its cost of equity is worth 1.0x tangible book value in this model. It is a way to read returns, not a price target. Not investment advice.</t>
+          <t>Justified P/TBV = (RoTE - g) / (CoE - g), with CoE 10% and g 2% as stated assumptions. No market prices are used. A bank that earns exactly its cost of equity is worth 1.0x tangible book value in this model. It is a way to read returns, not a price target. Not investment advice.</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="B45" s="86" t="inlineStr">
         <is>
-          <t>(RoTE − g) / (CoE − g)</t>
+          <t>(RoTE - g) / (CoE - g)</t>
         </is>
       </c>
       <c r="C45" s="86" t="n"/>
@@ -7798,7 +7798,7 @@
       <c r="C56" s="13" t="n"/>
       <c r="D56" s="14" t="n"/>
     </row>
-    <row r="57" ht="17.5" customHeight="1">
+    <row r="57" ht="31" customHeight="1">
       <c r="A57" s="28" t="inlineStr">
         <is>
           <t>CET1 ratios</t>
@@ -7806,7 +7806,7 @@
       </c>
       <c r="B57" s="85" t="inlineStr">
         <is>
-          <t>Include year-end profit net of the dividend accrual that each bank applies, so they are not perfectly comparable</t>
+          <t>As reported. NBG, Alpha and Piraeus include FY2024 profit (NBG and Alpha after a dividend provision); Eurobank's 16.8% is before its FY2024 dividend accrual (15.7% pro forma), so they are not perfectly comparable</t>
         </is>
       </c>
       <c r="C57" s="13" t="n"/>
@@ -7865,5 +7865,8 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="33" min="0" max="16383" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
</xml_diff>